<commit_message>
Daily NSE scan: 2026-10-05
</commit_message>
<xml_diff>
--- a/output/2026-10-05/enriched_analysis.xlsx
+++ b/output/2026-10-05/enriched_analysis.xlsx
@@ -929,13 +929,13 @@
         </is>
       </c>
       <c r="V2" t="n">
-        <v>2.204</v>
+        <v>2.188</v>
       </c>
       <c r="W2" t="n">
-        <v>2859</v>
+        <v>2880</v>
       </c>
       <c r="X2" t="n">
-        <v>22.4</v>
+        <v>22.5</v>
       </c>
       <c r="Y2" t="n">
         <v>75</v>
@@ -1161,13 +1161,13 @@
         </is>
       </c>
       <c r="V3" t="n">
-        <v>0.896</v>
+        <v>0.87</v>
       </c>
       <c r="W3" t="n">
-        <v>904</v>
+        <v>931</v>
       </c>
       <c r="X3" t="n">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="Y3" t="n">
         <v>47</v>
@@ -1393,13 +1393,13 @@
         </is>
       </c>
       <c r="V4" t="n">
-        <v>0.048</v>
+        <v>0.049</v>
       </c>
       <c r="W4" t="n">
-        <v>2766</v>
+        <v>2718</v>
       </c>
       <c r="X4" t="n">
-        <v>9.51</v>
+        <v>9.380000000000001</v>
       </c>
       <c r="Y4" t="n">
         <v>36</v>
@@ -1625,13 +1625,13 @@
         </is>
       </c>
       <c r="V5" t="n">
-        <v>1.124</v>
+        <v>1.138</v>
       </c>
       <c r="W5" t="n">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="X5" t="n">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="Y5" t="n">
         <v>22</v>
@@ -1857,13 +1857,13 @@
         </is>
       </c>
       <c r="V6" t="n">
-        <v>0.328</v>
+        <v>0.33</v>
       </c>
       <c r="W6" t="n">
-        <v>933</v>
+        <v>927</v>
       </c>
       <c r="X6" t="n">
-        <v>9.17</v>
+        <v>9.09</v>
       </c>
       <c r="Y6" t="n">
         <v>7</v>
@@ -2089,13 +2089,13 @@
         </is>
       </c>
       <c r="V7" t="n">
-        <v>1.013</v>
+        <v>1.019</v>
       </c>
       <c r="W7" t="n">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="X7" t="n">
-        <v>8.43</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="Y7" t="n">
         <v>17</v>
@@ -2321,13 +2321,13 @@
         </is>
       </c>
       <c r="V8" t="n">
-        <v>0.534</v>
+        <v>0.531</v>
       </c>
       <c r="W8" t="n">
-        <v>2673</v>
+        <v>2687</v>
       </c>
       <c r="X8" t="n">
-        <v>21.9</v>
+        <v>22</v>
       </c>
       <c r="Y8" t="n">
         <v>8</v>
@@ -2490,7 +2490,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F9" t="n">
         <v>5</v>
@@ -2553,10 +2553,10 @@
         </is>
       </c>
       <c r="V9" t="n">
-        <v>0.998</v>
+        <v>1.001</v>
       </c>
       <c r="W9" t="n">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="X9" t="inlineStr"/>
       <c r="Y9" t="n">
@@ -2783,13 +2783,13 @@
         </is>
       </c>
       <c r="V10" t="n">
-        <v>0.048</v>
+        <v>0.049</v>
       </c>
       <c r="W10" t="n">
-        <v>15109</v>
+        <v>14717</v>
       </c>
       <c r="X10" t="n">
-        <v>38.5</v>
+        <v>37.5</v>
       </c>
       <c r="Y10" t="n">
         <v>83</v>
@@ -3015,13 +3015,13 @@
         </is>
       </c>
       <c r="V11" t="n">
-        <v>0.125</v>
+        <v>0.128</v>
       </c>
       <c r="W11" t="n">
-        <v>2502</v>
+        <v>2452</v>
       </c>
       <c r="X11" t="n">
-        <v>21.9</v>
+        <v>21.5</v>
       </c>
       <c r="Y11" t="n">
         <v>-3</v>
@@ -3247,10 +3247,10 @@
         </is>
       </c>
       <c r="V12" t="n">
-        <v>2.286</v>
+        <v>2.288</v>
       </c>
       <c r="W12" t="n">
-        <v>2568</v>
+        <v>2565</v>
       </c>
       <c r="X12" t="n">
         <v>201</v>
@@ -3479,13 +3479,13 @@
         </is>
       </c>
       <c r="V13" t="n">
-        <v>0.124</v>
+        <v>0.128</v>
       </c>
       <c r="W13" t="n">
-        <v>692</v>
+        <v>669</v>
       </c>
       <c r="X13" t="n">
-        <v>30.1</v>
+        <v>29.2</v>
       </c>
       <c r="Y13" t="n">
         <v>17</v>
@@ -3705,13 +3705,13 @@
         </is>
       </c>
       <c r="V14" t="n">
-        <v>0.067</v>
+        <v>0.066</v>
       </c>
       <c r="W14" t="n">
-        <v>846</v>
+        <v>860</v>
       </c>
       <c r="X14" t="n">
-        <v>21.4</v>
+        <v>21.7</v>
       </c>
       <c r="Y14" t="n">
         <v>19</v>
@@ -3935,13 +3935,13 @@
         </is>
       </c>
       <c r="V15" t="n">
-        <v>0.049</v>
+        <v>0.051</v>
       </c>
       <c r="W15" t="n">
-        <v>1667</v>
+        <v>1624</v>
       </c>
       <c r="X15" t="n">
-        <v>22.5</v>
+        <v>21.9</v>
       </c>
       <c r="Y15" t="n">
         <v>55</v>
@@ -4170,10 +4170,10 @@
         <v>0.063</v>
       </c>
       <c r="W16" t="n">
-        <v>1759</v>
+        <v>1752</v>
       </c>
       <c r="X16" t="n">
-        <v>40.4</v>
+        <v>40.2</v>
       </c>
       <c r="Y16" t="n">
         <v>20</v>
@@ -4399,13 +4399,13 @@
         </is>
       </c>
       <c r="V17" t="n">
-        <v>2.848</v>
+        <v>2.783</v>
       </c>
       <c r="W17" t="n">
-        <v>691</v>
+        <v>707</v>
       </c>
       <c r="X17" t="n">
-        <v>26</v>
+        <v>26.6</v>
       </c>
       <c r="Y17" t="n">
         <v>30</v>
@@ -4625,13 +4625,13 @@
         </is>
       </c>
       <c r="V18" t="n">
-        <v>0.657</v>
+        <v>0.665</v>
       </c>
       <c r="W18" t="n">
-        <v>441</v>
+        <v>436</v>
       </c>
       <c r="X18" t="n">
-        <v>11</v>
+        <v>10.9</v>
       </c>
       <c r="Y18" t="n">
         <v>19</v>
@@ -4857,13 +4857,13 @@
         </is>
       </c>
       <c r="V19" t="n">
-        <v>0.325</v>
+        <v>0.334</v>
       </c>
       <c r="W19" t="n">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="X19" t="n">
-        <v>23.6</v>
+        <v>23</v>
       </c>
       <c r="Y19" t="n">
         <v>12</v>
@@ -4881,7 +4881,7 @@
         <v>7.91</v>
       </c>
       <c r="AD19" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AE19" t="b">
         <v>0</v>
@@ -5089,13 +5089,13 @@
         </is>
       </c>
       <c r="V20" t="n">
-        <v>0.371</v>
+        <v>0.376</v>
       </c>
       <c r="W20" t="n">
-        <v>1060</v>
+        <v>1047</v>
       </c>
       <c r="X20" t="n">
-        <v>54</v>
+        <v>53.4</v>
       </c>
       <c r="Y20" t="n">
         <v>21</v>
@@ -5324,10 +5324,10 @@
         <v>0.008999999999999999</v>
       </c>
       <c r="W21" t="n">
-        <v>52750</v>
+        <v>53385</v>
       </c>
       <c r="X21" t="n">
-        <v>44.7</v>
+        <v>45.2</v>
       </c>
       <c r="Y21" t="n">
         <v>5</v>
@@ -5553,13 +5553,13 @@
         </is>
       </c>
       <c r="V22" t="n">
-        <v>0.191</v>
+        <v>0.19</v>
       </c>
       <c r="W22" t="n">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="X22" t="n">
-        <v>48.5</v>
+        <v>48.6</v>
       </c>
       <c r="Y22" t="n">
         <v>3</v>
@@ -5577,7 +5577,7 @@
         <v>11.6</v>
       </c>
       <c r="AD22" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AE22" t="b">
         <v>1</v>
@@ -5785,13 +5785,13 @@
         </is>
       </c>
       <c r="V23" t="n">
-        <v>0.09</v>
+        <v>0.089</v>
       </c>
       <c r="W23" t="n">
-        <v>634</v>
+        <v>639</v>
       </c>
       <c r="X23" t="n">
-        <v>10.3</v>
+        <v>10.4</v>
       </c>
       <c r="Y23" t="n">
         <v>-5</v>
@@ -6017,13 +6017,13 @@
         </is>
       </c>
       <c r="V24" t="n">
-        <v>0.508</v>
+        <v>0.509</v>
       </c>
       <c r="W24" t="n">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="X24" t="n">
-        <v>36.5</v>
+        <v>36.4</v>
       </c>
       <c r="Y24" t="n">
         <v>21</v>
@@ -6249,13 +6249,13 @@
         </is>
       </c>
       <c r="V25" t="n">
-        <v>0.931</v>
+        <v>0.977</v>
       </c>
       <c r="W25" t="n">
-        <v>213</v>
+        <v>203</v>
       </c>
       <c r="X25" t="n">
-        <v>6.24</v>
+        <v>5.92</v>
       </c>
       <c r="Y25" t="n">
         <v>31</v>
@@ -6477,13 +6477,13 @@
         </is>
       </c>
       <c r="V26" t="n">
-        <v>0.275</v>
+        <v>0.289</v>
       </c>
       <c r="W26" t="n">
-        <v>948</v>
+        <v>899</v>
       </c>
       <c r="X26" t="n">
-        <v>25.8</v>
+        <v>24.5</v>
       </c>
       <c r="Y26" t="n">
         <v>9</v>
@@ -6709,13 +6709,13 @@
         </is>
       </c>
       <c r="V27" t="n">
-        <v>0.238</v>
+        <v>0.234</v>
       </c>
       <c r="W27" t="n">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="X27" t="n">
-        <v>14.3</v>
+        <v>14.6</v>
       </c>
       <c r="Y27" t="n">
         <v>16</v>
@@ -6941,13 +6941,13 @@
         </is>
       </c>
       <c r="V28" t="n">
-        <v>0.504</v>
+        <v>0.509</v>
       </c>
       <c r="W28" t="n">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="X28" t="n">
-        <v>36.9</v>
+        <v>36.5</v>
       </c>
       <c r="Y28" t="n">
         <v>-44</v>
@@ -7173,13 +7173,13 @@
         </is>
       </c>
       <c r="V29" t="n">
-        <v>0.133</v>
+        <v>0.134</v>
       </c>
       <c r="W29" t="n">
-        <v>602</v>
+        <v>598</v>
       </c>
       <c r="X29" t="n">
-        <v>13.3</v>
+        <v>13.2</v>
       </c>
       <c r="Y29" t="n">
         <v>-1</v>
@@ -7408,10 +7408,10 @@
         <v>0.044</v>
       </c>
       <c r="W30" t="n">
-        <v>1574</v>
+        <v>1585</v>
       </c>
       <c r="X30" t="n">
-        <v>20.6</v>
+        <v>20.7</v>
       </c>
       <c r="Y30" t="n">
         <v>10</v>
@@ -7637,13 +7637,13 @@
         </is>
       </c>
       <c r="V31" t="n">
-        <v>0.65</v>
+        <v>0.658</v>
       </c>
       <c r="W31" t="n">
-        <v>361</v>
+        <v>357</v>
       </c>
       <c r="X31" t="n">
-        <v>1164</v>
+        <v>1152</v>
       </c>
       <c r="Y31" t="n">
         <v>-61</v>
@@ -7865,13 +7865,13 @@
         </is>
       </c>
       <c r="V32" t="n">
-        <v>0.829</v>
+        <v>0.833</v>
       </c>
       <c r="W32" t="n">
-        <v>3810</v>
+        <v>3793</v>
       </c>
       <c r="X32" t="n">
-        <v>26.7</v>
+        <v>26.5</v>
       </c>
       <c r="Y32" t="n">
         <v>2</v>
@@ -8323,13 +8323,13 @@
         </is>
       </c>
       <c r="V34" t="n">
-        <v>0.366</v>
+        <v>0.371</v>
       </c>
       <c r="W34" t="n">
-        <v>383</v>
+        <v>377</v>
       </c>
       <c r="X34" t="n">
-        <v>94.7</v>
+        <v>93.3</v>
       </c>
       <c r="Y34" t="n">
         <v>246</v>
@@ -8555,10 +8555,10 @@
         </is>
       </c>
       <c r="V35" t="n">
-        <v>1.909</v>
+        <v>1.814</v>
       </c>
       <c r="W35" t="n">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="X35" t="inlineStr"/>
       <c r="Y35" t="n">
@@ -8785,13 +8785,13 @@
         </is>
       </c>
       <c r="V36" t="n">
-        <v>0.23</v>
+        <v>0.232</v>
       </c>
       <c r="W36" t="n">
-        <v>1733</v>
+        <v>1722</v>
       </c>
       <c r="X36" t="n">
-        <v>18.3</v>
+        <v>18.2</v>
       </c>
       <c r="Y36" t="n">
         <v>-3</v>
@@ -9020,10 +9020,10 @@
         <v>0.042</v>
       </c>
       <c r="W37" t="n">
-        <v>3230</v>
+        <v>3172</v>
       </c>
       <c r="X37" t="n">
-        <v>19.2</v>
+        <v>18.8</v>
       </c>
       <c r="Y37" t="n">
         <v>-4</v>
@@ -9252,7 +9252,7 @@
         <v>0.011</v>
       </c>
       <c r="W38" t="n">
-        <v>4187</v>
+        <v>4189</v>
       </c>
       <c r="X38" t="inlineStr"/>
       <c r="Y38" t="n">
@@ -9479,13 +9479,13 @@
         </is>
       </c>
       <c r="V39" t="n">
-        <v>0.114</v>
+        <v>0.109</v>
       </c>
       <c r="W39" t="n">
-        <v>435</v>
+        <v>456</v>
       </c>
       <c r="X39" t="n">
-        <v>7.02</v>
+        <v>7.3</v>
       </c>
       <c r="Y39" t="n">
         <v>118</v>
@@ -9710,7 +9710,7 @@
         <v>0</v>
       </c>
       <c r="W40" t="n">
-        <v>5001</v>
+        <v>4995</v>
       </c>
       <c r="X40" t="n">
         <v>11.7</v>
@@ -9939,13 +9939,13 @@
         </is>
       </c>
       <c r="V41" t="n">
-        <v>0.077</v>
+        <v>0.078</v>
       </c>
       <c r="W41" t="n">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="X41" t="n">
-        <v>12.9</v>
+        <v>12.8</v>
       </c>
       <c r="Y41" t="n">
         <v>-8</v>
@@ -10171,13 +10171,13 @@
         </is>
       </c>
       <c r="V42" t="n">
-        <v>0.119</v>
+        <v>0.125</v>
       </c>
       <c r="W42" t="n">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="X42" t="n">
-        <v>39.4</v>
+        <v>37.4</v>
       </c>
       <c r="Y42" t="n">
         <v>19</v>
@@ -10403,10 +10403,10 @@
         </is>
       </c>
       <c r="V43" t="n">
-        <v>0.052</v>
+        <v>0.053</v>
       </c>
       <c r="W43" t="n">
-        <v>954</v>
+        <v>938</v>
       </c>
       <c r="X43" t="inlineStr"/>
       <c r="Y43" t="n">
@@ -10633,13 +10633,13 @@
         </is>
       </c>
       <c r="V44" t="n">
-        <v>0.107</v>
+        <v>0.105</v>
       </c>
       <c r="W44" t="n">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="X44" t="n">
-        <v>25.6</v>
+        <v>26.1</v>
       </c>
       <c r="Y44" t="n">
         <v>24</v>
@@ -10868,10 +10868,10 @@
         <v>0.006</v>
       </c>
       <c r="W45" t="n">
-        <v>4951</v>
+        <v>4849</v>
       </c>
       <c r="X45" t="n">
-        <v>12.8</v>
+        <v>12.5</v>
       </c>
       <c r="Y45" t="n">
         <v>23</v>
@@ -11096,10 +11096,10 @@
         <v>0</v>
       </c>
       <c r="W46" t="n">
-        <v>3686</v>
+        <v>3776</v>
       </c>
       <c r="X46" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="Y46" t="n">
         <v>42</v>
@@ -11331,7 +11331,7 @@
         <v>206</v>
       </c>
       <c r="X47" t="n">
-        <v>24.6</v>
+        <v>24.5</v>
       </c>
       <c r="Y47" t="n">
         <v>21</v>
@@ -11560,10 +11560,10 @@
         <v>0</v>
       </c>
       <c r="W48" t="n">
-        <v>112261</v>
+        <v>111230</v>
       </c>
       <c r="X48" t="n">
-        <v>32.3</v>
+        <v>32</v>
       </c>
       <c r="Y48" t="n">
         <v>18</v>

</xml_diff>